<commit_message>
test: the Format Painter of Excel for Mac in paste-excel, 14 cases as Formats
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/paste/painter/onto-merged-formats.xlsx
+++ b/test/excel/paste/painter/onto-merged-formats.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mike/Library/Containers/com.microsoft.Excel/Data/tmp/fsave-48173/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mike/Library/Containers/com.microsoft.Excel/Data/tmp/fsave-50444/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EED76363-8B4A-9140-8FA0-48322E5691C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B6B72AFE-48DC-7741-B370-0067BAE3E72D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>